<commit_message>
Made FTU and NTU lowercase in conversions
</commit_message>
<xml_diff>
--- a/Meta/Analytes3.xlsx
+++ b/Meta/Analytes3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/vitense_kelsey_epa_gov/Documents/GL_Data/Meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="219" documentId="11_CFA7FA0AC8BEC675FF6906A82B7A2EC91D13FE60" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FAF63563-9F10-47A8-8CF6-A13C21A25AE4}"/>
+  <xr:revisionPtr revIDLastSave="238" documentId="11_CFA7FA0AC8BEC675FF6906A82B7A2EC91D13FE60" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E5D6A43-EF34-47DA-8DD4-B826B6962B6A}"/>
   <bookViews>
-    <workbookView xWindow="-61548" yWindow="-1872" windowWidth="30936" windowHeight="16776" tabRatio="802" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-61548" yWindow="-1872" windowWidth="30936" windowHeight="16776" tabRatio="802" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="11" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2711" uniqueCount="691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2711" uniqueCount="693">
   <si>
     <t>ANALYTE</t>
   </si>
@@ -2131,6 +2131,12 @@
   </si>
   <si>
     <t>PAR</t>
+  </si>
+  <si>
+    <t>ftu</t>
+  </si>
+  <si>
+    <t>ntu</t>
   </si>
 </sst>
 </file>
@@ -2611,35 +2617,11 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -2647,10 +2629,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2664,6 +2646,30 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8086,8 +8092,8 @@
       <c r="J2" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="K2" s="73"/>
-      <c r="L2" s="77"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="69"/>
       <c r="M2" s="24" t="s">
         <v>257</v>
       </c>
@@ -8124,8 +8130,8 @@
       <c r="J3" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K3" s="74"/>
-      <c r="L3" s="78"/>
+      <c r="K3" s="68"/>
+      <c r="L3" s="70"/>
       <c r="M3" s="9" t="s">
         <v>257</v>
       </c>
@@ -8162,8 +8168,8 @@
       <c r="J4" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K4" s="74"/>
-      <c r="L4" s="78"/>
+      <c r="K4" s="68"/>
+      <c r="L4" s="70"/>
       <c r="M4" s="9" t="s">
         <v>257</v>
       </c>
@@ -8198,8 +8204,8 @@
       <c r="J5" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K5" s="74"/>
-      <c r="L5" s="78"/>
+      <c r="K5" s="68"/>
+      <c r="L5" s="70"/>
       <c r="M5" s="9" t="s">
         <v>257</v>
       </c>
@@ -8236,10 +8242,10 @@
       <c r="J6" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K6" s="76" t="s">
+      <c r="K6" s="71" t="s">
         <v>267</v>
       </c>
-      <c r="L6" s="81"/>
+      <c r="L6" s="73"/>
       <c r="M6" s="9" t="s">
         <v>257</v>
       </c>
@@ -8276,8 +8282,8 @@
       <c r="J7" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K7" s="74"/>
-      <c r="L7" s="82"/>
+      <c r="K7" s="68"/>
+      <c r="L7" s="74"/>
       <c r="M7" s="9" t="s">
         <v>257</v>
       </c>
@@ -8312,8 +8318,8 @@
       <c r="J8" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K8" s="75"/>
-      <c r="L8" s="83"/>
+      <c r="K8" s="72"/>
+      <c r="L8" s="75"/>
       <c r="M8" s="9" t="s">
         <v>257</v>
       </c>
@@ -8350,10 +8356,10 @@
       <c r="J9" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K9" s="84" t="s">
+      <c r="K9" s="76" t="s">
         <v>275</v>
       </c>
-      <c r="L9" s="79" t="s">
+      <c r="L9" s="78" t="s">
         <v>276</v>
       </c>
       <c r="M9" s="24" t="s">
@@ -8392,8 +8398,8 @@
       <c r="J10" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K10" s="68"/>
-      <c r="L10" s="78"/>
+      <c r="K10" s="77"/>
+      <c r="L10" s="70"/>
       <c r="M10" s="9" t="s">
         <v>257</v>
       </c>
@@ -8430,8 +8436,8 @@
       <c r="J11" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K11" s="68"/>
-      <c r="L11" s="78"/>
+      <c r="K11" s="77"/>
+      <c r="L11" s="70"/>
       <c r="M11" s="9" t="s">
         <v>257</v>
       </c>
@@ -8710,7 +8716,7 @@
       <c r="J18" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K18" s="76"/>
+      <c r="K18" s="71"/>
       <c r="L18" s="22"/>
       <c r="M18" s="9" t="s">
         <v>257</v>
@@ -8748,7 +8754,7 @@
       <c r="J19" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K19" s="75"/>
+      <c r="K19" s="72"/>
       <c r="L19" s="44"/>
       <c r="M19" s="27" t="s">
         <v>257</v>
@@ -8786,10 +8792,10 @@
       <c r="J20" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K20" s="76" t="s">
+      <c r="K20" s="71" t="s">
         <v>310</v>
       </c>
-      <c r="L20" s="79" t="s">
+      <c r="L20" s="78" t="s">
         <v>311</v>
       </c>
       <c r="M20" s="9" t="s">
@@ -8828,8 +8834,8 @@
       <c r="J21" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K21" s="74"/>
-      <c r="L21" s="78"/>
+      <c r="K21" s="68"/>
+      <c r="L21" s="70"/>
       <c r="M21" s="9" t="s">
         <v>257</v>
       </c>
@@ -8864,8 +8870,8 @@
       <c r="J22" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K22" s="74"/>
-      <c r="L22" s="78"/>
+      <c r="K22" s="68"/>
+      <c r="L22" s="70"/>
       <c r="M22" s="9" t="s">
         <v>257</v>
       </c>
@@ -8902,8 +8908,8 @@
       <c r="J23" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K23" s="74"/>
-      <c r="L23" s="78"/>
+      <c r="K23" s="68"/>
+      <c r="L23" s="70"/>
       <c r="M23" s="9" t="s">
         <v>257</v>
       </c>
@@ -8940,8 +8946,8 @@
       <c r="J24" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K24" s="74"/>
-      <c r="L24" s="78"/>
+      <c r="K24" s="68"/>
+      <c r="L24" s="70"/>
       <c r="M24" s="9" t="s">
         <v>257</v>
       </c>
@@ -8978,10 +8984,10 @@
       <c r="J25" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="K25" s="73" t="s">
+      <c r="K25" s="67" t="s">
         <v>317</v>
       </c>
-      <c r="L25" s="77" t="s">
+      <c r="L25" s="69" t="s">
         <v>318</v>
       </c>
       <c r="M25" s="24" t="s">
@@ -9020,8 +9026,8 @@
       <c r="J26" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K26" s="74"/>
-      <c r="L26" s="78"/>
+      <c r="K26" s="68"/>
+      <c r="L26" s="70"/>
       <c r="M26" s="9" t="s">
         <v>257</v>
       </c>
@@ -9058,8 +9064,8 @@
       <c r="J27" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K27" s="74"/>
-      <c r="L27" s="78"/>
+      <c r="K27" s="68"/>
+      <c r="L27" s="70"/>
       <c r="M27" s="9" t="s">
         <v>257</v>
       </c>
@@ -9094,8 +9100,8 @@
       <c r="J28" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K28" s="75"/>
-      <c r="L28" s="80"/>
+      <c r="K28" s="72"/>
+      <c r="L28" s="79"/>
       <c r="M28" s="27" t="s">
         <v>257</v>
       </c>
@@ -9132,7 +9138,7 @@
       <c r="J29" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K29" s="76" t="s">
+      <c r="K29" s="71" t="s">
         <v>323</v>
       </c>
       <c r="L29" s="22"/>
@@ -9172,7 +9178,7 @@
       <c r="J30" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K30" s="74"/>
+      <c r="K30" s="68"/>
       <c r="L30" s="22"/>
       <c r="M30" s="9" t="s">
         <v>257</v>
@@ -9210,7 +9216,7 @@
       <c r="J31" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K31" s="74"/>
+      <c r="K31" s="68"/>
       <c r="L31" s="22"/>
       <c r="M31" s="9" t="s">
         <v>257</v>
@@ -9246,7 +9252,7 @@
       <c r="J32" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K32" s="74"/>
+      <c r="K32" s="68"/>
       <c r="L32" s="22"/>
       <c r="M32" s="9" t="s">
         <v>257</v>
@@ -9284,7 +9290,7 @@
       <c r="J33" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="K33" s="73" t="s">
+      <c r="K33" s="67" t="s">
         <v>290</v>
       </c>
       <c r="L33" s="43" t="s">
@@ -9326,7 +9332,7 @@
       <c r="J34" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K34" s="75"/>
+      <c r="K34" s="72"/>
       <c r="L34" s="44"/>
       <c r="M34" s="27" t="s">
         <v>257</v>
@@ -9364,7 +9370,7 @@
       <c r="J35" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K35" s="76" t="s">
+      <c r="K35" s="71" t="s">
         <v>290</v>
       </c>
       <c r="L35" s="22" t="s">
@@ -9406,7 +9412,7 @@
       <c r="J36" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K36" s="74"/>
+      <c r="K36" s="68"/>
       <c r="L36" s="22"/>
       <c r="M36" s="9" t="s">
         <v>257</v>
@@ -9523,7 +9529,7 @@
       <c r="K39" s="46" t="s">
         <v>340</v>
       </c>
-      <c r="L39" s="77"/>
+      <c r="L39" s="69"/>
       <c r="M39" s="24" t="s">
         <v>257</v>
       </c>
@@ -9561,7 +9567,7 @@
         <v>257</v>
       </c>
       <c r="K40" s="35"/>
-      <c r="L40" s="78"/>
+      <c r="L40" s="70"/>
       <c r="M40" s="9" t="s">
         <v>257</v>
       </c>
@@ -9640,10 +9646,10 @@
       <c r="J42" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K42" s="76" t="s">
+      <c r="K42" s="71" t="s">
         <v>347</v>
       </c>
-      <c r="L42" s="79" t="s">
+      <c r="L42" s="78" t="s">
         <v>348</v>
       </c>
       <c r="M42" s="24" t="s">
@@ -9682,8 +9688,8 @@
       <c r="J43" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K43" s="74"/>
-      <c r="L43" s="78"/>
+      <c r="K43" s="68"/>
+      <c r="L43" s="70"/>
       <c r="M43" s="9" t="s">
         <v>257</v>
       </c>
@@ -9720,8 +9726,8 @@
       <c r="J44" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K44" s="74"/>
-      <c r="L44" s="78"/>
+      <c r="K44" s="68"/>
+      <c r="L44" s="70"/>
       <c r="M44" s="9" t="s">
         <v>257</v>
       </c>
@@ -9756,8 +9762,8 @@
       <c r="J45" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K45" s="74"/>
-      <c r="L45" s="78"/>
+      <c r="K45" s="68"/>
+      <c r="L45" s="70"/>
       <c r="M45" s="9" t="s">
         <v>257</v>
       </c>
@@ -9794,8 +9800,8 @@
       <c r="J46" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K46" s="74"/>
-      <c r="L46" s="78"/>
+      <c r="K46" s="68"/>
+      <c r="L46" s="70"/>
       <c r="M46" s="9" t="s">
         <v>257</v>
       </c>
@@ -9832,8 +9838,8 @@
       <c r="J47" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K47" s="74"/>
-      <c r="L47" s="78"/>
+      <c r="K47" s="68"/>
+      <c r="L47" s="70"/>
       <c r="M47" s="9" t="s">
         <v>257</v>
       </c>
@@ -9950,7 +9956,7 @@
       <c r="J50" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="K50" s="67" t="s">
+      <c r="K50" s="80" t="s">
         <v>361</v>
       </c>
       <c r="L50" s="43"/>
@@ -9990,7 +9996,7 @@
       <c r="J51" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K51" s="68"/>
+      <c r="K51" s="77"/>
       <c r="L51" s="22"/>
       <c r="M51" s="24" t="s">
         <v>257</v>
@@ -10028,7 +10034,7 @@
       <c r="J52" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K52" s="68"/>
+      <c r="K52" s="77"/>
       <c r="L52" s="22"/>
       <c r="M52" s="24" t="s">
         <v>257</v>
@@ -10066,7 +10072,7 @@
       <c r="J53" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K53" s="68"/>
+      <c r="K53" s="77"/>
       <c r="L53" s="22"/>
       <c r="M53" s="24" t="s">
         <v>257</v>
@@ -10102,7 +10108,7 @@
       <c r="J54" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K54" s="69"/>
+      <c r="K54" s="81"/>
       <c r="L54" s="44"/>
       <c r="M54" s="24" t="s">
         <v>257</v>
@@ -10222,7 +10228,7 @@
       <c r="J57" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K57" s="76" t="s">
+      <c r="K57" s="71" t="s">
         <v>378</v>
       </c>
       <c r="L57" s="22"/>
@@ -10262,7 +10268,7 @@
       <c r="J58" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K58" s="74"/>
+      <c r="K58" s="68"/>
       <c r="L58" s="22"/>
       <c r="M58" s="9" t="s">
         <v>257</v>
@@ -10298,7 +10304,7 @@
       <c r="J59" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K59" s="74"/>
+      <c r="K59" s="68"/>
       <c r="L59" s="22"/>
       <c r="M59" s="9" t="s">
         <v>257</v>
@@ -10336,7 +10342,7 @@
       <c r="J60" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="K60" s="77" t="s">
+      <c r="K60" s="69" t="s">
         <v>383</v>
       </c>
       <c r="L60" s="43"/>
@@ -10376,7 +10382,7 @@
       <c r="J61" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="K61" s="78"/>
+      <c r="K61" s="70"/>
       <c r="L61" s="22" t="s">
         <v>385</v>
       </c>
@@ -10416,7 +10422,7 @@
       <c r="J62" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K62" s="78"/>
+      <c r="K62" s="70"/>
       <c r="L62" s="22" t="s">
         <v>387</v>
       </c>
@@ -10456,7 +10462,7 @@
       <c r="J63" s="47" t="s">
         <v>257</v>
       </c>
-      <c r="K63" s="76"/>
+      <c r="K63" s="71"/>
       <c r="L63" s="22"/>
       <c r="M63" s="9" t="s">
         <v>257</v>
@@ -10494,7 +10500,7 @@
       <c r="J64" s="47" t="s">
         <v>257</v>
       </c>
-      <c r="K64" s="74"/>
+      <c r="K64" s="68"/>
       <c r="L64" s="22"/>
       <c r="M64" s="9" t="s">
         <v>257</v>
@@ -10532,7 +10538,7 @@
       <c r="J65" s="47" t="s">
         <v>257</v>
       </c>
-      <c r="K65" s="74"/>
+      <c r="K65" s="68"/>
       <c r="L65" s="22" t="s">
         <v>387</v>
       </c>
@@ -10570,7 +10576,7 @@
       <c r="J66" s="47" t="s">
         <v>257</v>
       </c>
-      <c r="K66" s="74"/>
+      <c r="K66" s="68"/>
       <c r="L66" s="13"/>
       <c r="M66" s="34" t="s">
         <v>257</v>
@@ -10684,7 +10690,7 @@
       <c r="J69" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K69" s="76" t="s">
+      <c r="K69" s="71" t="s">
         <v>290</v>
       </c>
       <c r="L69" s="22" t="s">
@@ -10726,7 +10732,7 @@
       <c r="J70" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K70" s="74"/>
+      <c r="K70" s="68"/>
       <c r="L70" s="22"/>
       <c r="M70" s="9" t="s">
         <v>257</v>
@@ -10804,7 +10810,7 @@
       <c r="J72" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K72" s="76"/>
+      <c r="K72" s="71"/>
       <c r="L72" s="22"/>
       <c r="M72" s="9" t="s">
         <v>257</v>
@@ -10840,7 +10846,7 @@
       <c r="J73" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K73" s="74"/>
+      <c r="K73" s="68"/>
       <c r="L73" s="22"/>
       <c r="M73" s="9" t="s">
         <v>257</v>
@@ -10876,7 +10882,7 @@
       <c r="J74" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K74" s="74"/>
+      <c r="K74" s="68"/>
       <c r="L74" s="22"/>
       <c r="M74" s="9" t="s">
         <v>257</v>
@@ -10910,7 +10916,7 @@
       <c r="J75" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K75" s="75"/>
+      <c r="K75" s="72"/>
       <c r="L75" s="44"/>
       <c r="M75" s="9" t="s">
         <v>257</v>
@@ -10988,10 +10994,10 @@
       <c r="J77" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="K77" s="67" t="s">
+      <c r="K77" s="80" t="s">
         <v>410</v>
       </c>
-      <c r="L77" s="73" t="s">
+      <c r="L77" s="67" t="s">
         <v>411</v>
       </c>
       <c r="M77" s="24" t="s">
@@ -11032,8 +11038,8 @@
       <c r="J78" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K78" s="69"/>
-      <c r="L78" s="71"/>
+      <c r="K78" s="81"/>
+      <c r="L78" s="83"/>
       <c r="M78" s="34" t="s">
         <v>257</v>
       </c>
@@ -11073,7 +11079,7 @@
       <c r="K79" s="22" t="s">
         <v>412</v>
       </c>
-      <c r="L79" s="71"/>
+      <c r="L79" s="83"/>
       <c r="M79" s="34" t="s">
         <v>257</v>
       </c>
@@ -11113,7 +11119,7 @@
       <c r="K80" s="22" t="s">
         <v>412</v>
       </c>
-      <c r="L80" s="75"/>
+      <c r="L80" s="72"/>
       <c r="M80" s="9" t="s">
         <v>257</v>
       </c>
@@ -11150,7 +11156,7 @@
       <c r="J81" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K81" s="76" t="s">
+      <c r="K81" s="71" t="s">
         <v>290</v>
       </c>
       <c r="L81" s="22" t="s">
@@ -11192,7 +11198,7 @@
       <c r="J82" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K82" s="74"/>
+      <c r="K82" s="68"/>
       <c r="L82" s="22"/>
       <c r="M82" s="9" t="s">
         <v>257</v>
@@ -11314,7 +11320,7 @@
       <c r="J85" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K85" s="76" t="s">
+      <c r="K85" s="71" t="s">
         <v>424</v>
       </c>
       <c r="L85" s="22"/>
@@ -11354,7 +11360,7 @@
       <c r="J86" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K86" s="74"/>
+      <c r="K86" s="68"/>
       <c r="L86" s="22"/>
       <c r="M86" s="9" t="s">
         <v>257</v>
@@ -11392,7 +11398,7 @@
       <c r="J87" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K87" s="74"/>
+      <c r="K87" s="68"/>
       <c r="L87" s="22"/>
       <c r="M87" s="9" t="s">
         <v>257</v>
@@ -11428,7 +11434,7 @@
       <c r="J88" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K88" s="74"/>
+      <c r="K88" s="68"/>
       <c r="L88" s="22"/>
       <c r="M88" s="9" t="s">
         <v>257</v>
@@ -11466,7 +11472,7 @@
       <c r="J89" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K89" s="74"/>
+      <c r="K89" s="68"/>
       <c r="L89" s="22"/>
       <c r="M89" s="9" t="s">
         <v>257</v>
@@ -11504,7 +11510,7 @@
       <c r="J90" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K90" s="74"/>
+      <c r="K90" s="68"/>
       <c r="L90" s="22"/>
       <c r="M90" s="9" t="s">
         <v>257</v>
@@ -11542,10 +11548,10 @@
       <c r="J91" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K91" s="67" t="s">
+      <c r="K91" s="80" t="s">
         <v>430</v>
       </c>
-      <c r="L91" s="70" t="s">
+      <c r="L91" s="82" t="s">
         <v>431</v>
       </c>
       <c r="M91" s="24" t="s">
@@ -11584,8 +11590,8 @@
       <c r="J92" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="K92" s="68"/>
-      <c r="L92" s="71"/>
+      <c r="K92" s="77"/>
+      <c r="L92" s="83"/>
       <c r="M92" s="9" t="s">
         <v>257</v>
       </c>
@@ -11622,8 +11628,8 @@
       <c r="J93" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="K93" s="68"/>
-      <c r="L93" s="71"/>
+      <c r="K93" s="77"/>
+      <c r="L93" s="83"/>
       <c r="M93" s="9" t="s">
         <v>257</v>
       </c>
@@ -11658,8 +11664,8 @@
       <c r="J94" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K94" s="69"/>
-      <c r="L94" s="72"/>
+      <c r="K94" s="81"/>
+      <c r="L94" s="84"/>
       <c r="M94" s="9" t="s">
         <v>257</v>
       </c>
@@ -11696,7 +11702,7 @@
       <c r="J95" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K95" s="73"/>
+      <c r="K95" s="67"/>
       <c r="L95" s="22"/>
       <c r="M95" s="24" t="s">
         <v>257</v>
@@ -11734,7 +11740,7 @@
       <c r="J96" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K96" s="74"/>
+      <c r="K96" s="68"/>
       <c r="L96" s="22"/>
       <c r="M96" s="24" t="s">
         <v>257</v>
@@ -11772,7 +11778,7 @@
       <c r="J97" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K97" s="74"/>
+      <c r="K97" s="68"/>
       <c r="L97" s="22"/>
       <c r="M97" s="24" t="s">
         <v>257</v>
@@ -11810,7 +11816,7 @@
       <c r="J98" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K98" s="74"/>
+      <c r="K98" s="68"/>
       <c r="L98" s="22"/>
       <c r="M98" s="24" t="s">
         <v>257</v>
@@ -11846,7 +11852,7 @@
       <c r="J99" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K99" s="75"/>
+      <c r="K99" s="72"/>
       <c r="L99" s="37"/>
       <c r="M99" s="39" t="s">
         <v>257</v>
@@ -11875,28 +11881,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="K2:K5"/>
-    <mergeCell ref="L2:L5"/>
-    <mergeCell ref="K6:K8"/>
-    <mergeCell ref="L6:L8"/>
-    <mergeCell ref="K9:K11"/>
-    <mergeCell ref="L9:L11"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="K20:K24"/>
-    <mergeCell ref="L20:L24"/>
-    <mergeCell ref="K25:K28"/>
-    <mergeCell ref="L25:L28"/>
-    <mergeCell ref="K29:K32"/>
-    <mergeCell ref="K33:K34"/>
-    <mergeCell ref="K35:K36"/>
-    <mergeCell ref="L39:L40"/>
-    <mergeCell ref="K42:K47"/>
-    <mergeCell ref="L42:L47"/>
-    <mergeCell ref="K50:K54"/>
-    <mergeCell ref="K57:K59"/>
-    <mergeCell ref="K60:K62"/>
-    <mergeCell ref="K63:K66"/>
-    <mergeCell ref="K69:K70"/>
     <mergeCell ref="K91:K94"/>
     <mergeCell ref="L91:L94"/>
     <mergeCell ref="K95:K99"/>
@@ -11905,6 +11889,28 @@
     <mergeCell ref="L77:L80"/>
     <mergeCell ref="K81:K82"/>
     <mergeCell ref="K85:K90"/>
+    <mergeCell ref="K50:K54"/>
+    <mergeCell ref="K57:K59"/>
+    <mergeCell ref="K60:K62"/>
+    <mergeCell ref="K63:K66"/>
+    <mergeCell ref="K69:K70"/>
+    <mergeCell ref="K29:K32"/>
+    <mergeCell ref="K33:K34"/>
+    <mergeCell ref="K35:K36"/>
+    <mergeCell ref="L39:L40"/>
+    <mergeCell ref="K42:K47"/>
+    <mergeCell ref="L42:L47"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="K20:K24"/>
+    <mergeCell ref="L20:L24"/>
+    <mergeCell ref="K25:K28"/>
+    <mergeCell ref="L25:L28"/>
+    <mergeCell ref="K2:K5"/>
+    <mergeCell ref="L2:L5"/>
+    <mergeCell ref="K6:K8"/>
+    <mergeCell ref="L6:L8"/>
+    <mergeCell ref="K9:K11"/>
+    <mergeCell ref="L9:L11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14820,10 +14826,10 @@
     </row>
     <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>154</v>
+        <v>691</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>155</v>
+        <v>692</v>
       </c>
       <c r="C2" s="65" t="s">
         <v>12</v>
@@ -14876,10 +14882,10 @@
     </row>
     <row r="6" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>155</v>
+        <v>692</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>154</v>
+        <v>691</v>
       </c>
       <c r="C6" s="65" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Minor update to Analytes3
</commit_message>
<xml_diff>
--- a/Meta/Analytes3.xlsx
+++ b/Meta/Analytes3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/vitense_kelsey_epa_gov/Documents/GL_Data/Meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="238" documentId="11_CFA7FA0AC8BEC675FF6906A82B7A2EC91D13FE60" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E5D6A43-EF34-47DA-8DD4-B826B6962B6A}"/>
+  <xr:revisionPtr revIDLastSave="241" documentId="11_CFA7FA0AC8BEC675FF6906A82B7A2EC91D13FE60" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0C1EC90-6557-4C8E-BDFB-3B17394C2A46}"/>
   <bookViews>
-    <workbookView xWindow="-61548" yWindow="-1872" windowWidth="30936" windowHeight="16776" tabRatio="802" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-61548" yWindow="-1872" windowWidth="30936" windowHeight="16776" tabRatio="802" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="11" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2711" uniqueCount="693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2712" uniqueCount="695">
   <si>
     <t>ANALYTE</t>
   </si>
@@ -2137,6 +2137,12 @@
   </si>
   <si>
     <t>ntu</t>
+  </si>
+  <si>
+    <t>Note that all rows with Methods in this spreadsheet came from non-GL lakes. GL lake Methods are NA for all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">These are derived variables in code (from nitrate and nitrite). </t>
   </si>
 </sst>
 </file>
@@ -2617,11 +2623,35 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -2629,10 +2659,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2646,30 +2676,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8092,8 +8098,8 @@
       <c r="J2" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="K2" s="67"/>
-      <c r="L2" s="69"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="77"/>
       <c r="M2" s="24" t="s">
         <v>257</v>
       </c>
@@ -8130,8 +8136,8 @@
       <c r="J3" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K3" s="68"/>
-      <c r="L3" s="70"/>
+      <c r="K3" s="74"/>
+      <c r="L3" s="78"/>
       <c r="M3" s="9" t="s">
         <v>257</v>
       </c>
@@ -8168,8 +8174,8 @@
       <c r="J4" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K4" s="68"/>
-      <c r="L4" s="70"/>
+      <c r="K4" s="74"/>
+      <c r="L4" s="78"/>
       <c r="M4" s="9" t="s">
         <v>257</v>
       </c>
@@ -8204,8 +8210,8 @@
       <c r="J5" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K5" s="68"/>
-      <c r="L5" s="70"/>
+      <c r="K5" s="74"/>
+      <c r="L5" s="78"/>
       <c r="M5" s="9" t="s">
         <v>257</v>
       </c>
@@ -8242,10 +8248,10 @@
       <c r="J6" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K6" s="71" t="s">
+      <c r="K6" s="76" t="s">
         <v>267</v>
       </c>
-      <c r="L6" s="73"/>
+      <c r="L6" s="81"/>
       <c r="M6" s="9" t="s">
         <v>257</v>
       </c>
@@ -8282,8 +8288,8 @@
       <c r="J7" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K7" s="68"/>
-      <c r="L7" s="74"/>
+      <c r="K7" s="74"/>
+      <c r="L7" s="82"/>
       <c r="M7" s="9" t="s">
         <v>257</v>
       </c>
@@ -8318,8 +8324,8 @@
       <c r="J8" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K8" s="72"/>
-      <c r="L8" s="75"/>
+      <c r="K8" s="75"/>
+      <c r="L8" s="83"/>
       <c r="M8" s="9" t="s">
         <v>257</v>
       </c>
@@ -8356,10 +8362,10 @@
       <c r="J9" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K9" s="76" t="s">
+      <c r="K9" s="84" t="s">
         <v>275</v>
       </c>
-      <c r="L9" s="78" t="s">
+      <c r="L9" s="79" t="s">
         <v>276</v>
       </c>
       <c r="M9" s="24" t="s">
@@ -8398,8 +8404,8 @@
       <c r="J10" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K10" s="77"/>
-      <c r="L10" s="70"/>
+      <c r="K10" s="68"/>
+      <c r="L10" s="78"/>
       <c r="M10" s="9" t="s">
         <v>257</v>
       </c>
@@ -8436,8 +8442,8 @@
       <c r="J11" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K11" s="77"/>
-      <c r="L11" s="70"/>
+      <c r="K11" s="68"/>
+      <c r="L11" s="78"/>
       <c r="M11" s="9" t="s">
         <v>257</v>
       </c>
@@ -8716,7 +8722,7 @@
       <c r="J18" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K18" s="71"/>
+      <c r="K18" s="76"/>
       <c r="L18" s="22"/>
       <c r="M18" s="9" t="s">
         <v>257</v>
@@ -8754,7 +8760,7 @@
       <c r="J19" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K19" s="72"/>
+      <c r="K19" s="75"/>
       <c r="L19" s="44"/>
       <c r="M19" s="27" t="s">
         <v>257</v>
@@ -8792,10 +8798,10 @@
       <c r="J20" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K20" s="71" t="s">
+      <c r="K20" s="76" t="s">
         <v>310</v>
       </c>
-      <c r="L20" s="78" t="s">
+      <c r="L20" s="79" t="s">
         <v>311</v>
       </c>
       <c r="M20" s="9" t="s">
@@ -8834,8 +8840,8 @@
       <c r="J21" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K21" s="68"/>
-      <c r="L21" s="70"/>
+      <c r="K21" s="74"/>
+      <c r="L21" s="78"/>
       <c r="M21" s="9" t="s">
         <v>257</v>
       </c>
@@ -8870,8 +8876,8 @@
       <c r="J22" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K22" s="68"/>
-      <c r="L22" s="70"/>
+      <c r="K22" s="74"/>
+      <c r="L22" s="78"/>
       <c r="M22" s="9" t="s">
         <v>257</v>
       </c>
@@ -8908,8 +8914,8 @@
       <c r="J23" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K23" s="68"/>
-      <c r="L23" s="70"/>
+      <c r="K23" s="74"/>
+      <c r="L23" s="78"/>
       <c r="M23" s="9" t="s">
         <v>257</v>
       </c>
@@ -8946,8 +8952,8 @@
       <c r="J24" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K24" s="68"/>
-      <c r="L24" s="70"/>
+      <c r="K24" s="74"/>
+      <c r="L24" s="78"/>
       <c r="M24" s="9" t="s">
         <v>257</v>
       </c>
@@ -8984,10 +8990,10 @@
       <c r="J25" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="K25" s="67" t="s">
+      <c r="K25" s="73" t="s">
         <v>317</v>
       </c>
-      <c r="L25" s="69" t="s">
+      <c r="L25" s="77" t="s">
         <v>318</v>
       </c>
       <c r="M25" s="24" t="s">
@@ -9026,8 +9032,8 @@
       <c r="J26" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K26" s="68"/>
-      <c r="L26" s="70"/>
+      <c r="K26" s="74"/>
+      <c r="L26" s="78"/>
       <c r="M26" s="9" t="s">
         <v>257</v>
       </c>
@@ -9064,8 +9070,8 @@
       <c r="J27" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K27" s="68"/>
-      <c r="L27" s="70"/>
+      <c r="K27" s="74"/>
+      <c r="L27" s="78"/>
       <c r="M27" s="9" t="s">
         <v>257</v>
       </c>
@@ -9100,8 +9106,8 @@
       <c r="J28" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K28" s="72"/>
-      <c r="L28" s="79"/>
+      <c r="K28" s="75"/>
+      <c r="L28" s="80"/>
       <c r="M28" s="27" t="s">
         <v>257</v>
       </c>
@@ -9138,7 +9144,7 @@
       <c r="J29" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K29" s="71" t="s">
+      <c r="K29" s="76" t="s">
         <v>323</v>
       </c>
       <c r="L29" s="22"/>
@@ -9178,7 +9184,7 @@
       <c r="J30" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K30" s="68"/>
+      <c r="K30" s="74"/>
       <c r="L30" s="22"/>
       <c r="M30" s="9" t="s">
         <v>257</v>
@@ -9216,7 +9222,7 @@
       <c r="J31" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K31" s="68"/>
+      <c r="K31" s="74"/>
       <c r="L31" s="22"/>
       <c r="M31" s="9" t="s">
         <v>257</v>
@@ -9252,7 +9258,7 @@
       <c r="J32" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K32" s="68"/>
+      <c r="K32" s="74"/>
       <c r="L32" s="22"/>
       <c r="M32" s="9" t="s">
         <v>257</v>
@@ -9290,7 +9296,7 @@
       <c r="J33" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="K33" s="67" t="s">
+      <c r="K33" s="73" t="s">
         <v>290</v>
       </c>
       <c r="L33" s="43" t="s">
@@ -9332,7 +9338,7 @@
       <c r="J34" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K34" s="72"/>
+      <c r="K34" s="75"/>
       <c r="L34" s="44"/>
       <c r="M34" s="27" t="s">
         <v>257</v>
@@ -9370,7 +9376,7 @@
       <c r="J35" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K35" s="71" t="s">
+      <c r="K35" s="76" t="s">
         <v>290</v>
       </c>
       <c r="L35" s="22" t="s">
@@ -9412,7 +9418,7 @@
       <c r="J36" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K36" s="68"/>
+      <c r="K36" s="74"/>
       <c r="L36" s="22"/>
       <c r="M36" s="9" t="s">
         <v>257</v>
@@ -9529,7 +9535,7 @@
       <c r="K39" s="46" t="s">
         <v>340</v>
       </c>
-      <c r="L39" s="69"/>
+      <c r="L39" s="77"/>
       <c r="M39" s="24" t="s">
         <v>257</v>
       </c>
@@ -9567,7 +9573,7 @@
         <v>257</v>
       </c>
       <c r="K40" s="35"/>
-      <c r="L40" s="70"/>
+      <c r="L40" s="78"/>
       <c r="M40" s="9" t="s">
         <v>257</v>
       </c>
@@ -9646,10 +9652,10 @@
       <c r="J42" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K42" s="71" t="s">
+      <c r="K42" s="76" t="s">
         <v>347</v>
       </c>
-      <c r="L42" s="78" t="s">
+      <c r="L42" s="79" t="s">
         <v>348</v>
       </c>
       <c r="M42" s="24" t="s">
@@ -9688,8 +9694,8 @@
       <c r="J43" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K43" s="68"/>
-      <c r="L43" s="70"/>
+      <c r="K43" s="74"/>
+      <c r="L43" s="78"/>
       <c r="M43" s="9" t="s">
         <v>257</v>
       </c>
@@ -9726,8 +9732,8 @@
       <c r="J44" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K44" s="68"/>
-      <c r="L44" s="70"/>
+      <c r="K44" s="74"/>
+      <c r="L44" s="78"/>
       <c r="M44" s="9" t="s">
         <v>257</v>
       </c>
@@ -9762,8 +9768,8 @@
       <c r="J45" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K45" s="68"/>
-      <c r="L45" s="70"/>
+      <c r="K45" s="74"/>
+      <c r="L45" s="78"/>
       <c r="M45" s="9" t="s">
         <v>257</v>
       </c>
@@ -9800,8 +9806,8 @@
       <c r="J46" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K46" s="68"/>
-      <c r="L46" s="70"/>
+      <c r="K46" s="74"/>
+      <c r="L46" s="78"/>
       <c r="M46" s="9" t="s">
         <v>257</v>
       </c>
@@ -9838,8 +9844,8 @@
       <c r="J47" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K47" s="68"/>
-      <c r="L47" s="70"/>
+      <c r="K47" s="74"/>
+      <c r="L47" s="78"/>
       <c r="M47" s="9" t="s">
         <v>257</v>
       </c>
@@ -9956,7 +9962,7 @@
       <c r="J50" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="K50" s="80" t="s">
+      <c r="K50" s="67" t="s">
         <v>361</v>
       </c>
       <c r="L50" s="43"/>
@@ -9996,7 +10002,7 @@
       <c r="J51" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K51" s="77"/>
+      <c r="K51" s="68"/>
       <c r="L51" s="22"/>
       <c r="M51" s="24" t="s">
         <v>257</v>
@@ -10034,7 +10040,7 @@
       <c r="J52" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K52" s="77"/>
+      <c r="K52" s="68"/>
       <c r="L52" s="22"/>
       <c r="M52" s="24" t="s">
         <v>257</v>
@@ -10072,7 +10078,7 @@
       <c r="J53" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K53" s="77"/>
+      <c r="K53" s="68"/>
       <c r="L53" s="22"/>
       <c r="M53" s="24" t="s">
         <v>257</v>
@@ -10108,7 +10114,7 @@
       <c r="J54" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K54" s="81"/>
+      <c r="K54" s="69"/>
       <c r="L54" s="44"/>
       <c r="M54" s="24" t="s">
         <v>257</v>
@@ -10228,7 +10234,7 @@
       <c r="J57" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K57" s="71" t="s">
+      <c r="K57" s="76" t="s">
         <v>378</v>
       </c>
       <c r="L57" s="22"/>
@@ -10268,7 +10274,7 @@
       <c r="J58" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K58" s="68"/>
+      <c r="K58" s="74"/>
       <c r="L58" s="22"/>
       <c r="M58" s="9" t="s">
         <v>257</v>
@@ -10304,7 +10310,7 @@
       <c r="J59" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K59" s="68"/>
+      <c r="K59" s="74"/>
       <c r="L59" s="22"/>
       <c r="M59" s="9" t="s">
         <v>257</v>
@@ -10342,7 +10348,7 @@
       <c r="J60" s="24" t="s">
         <v>257</v>
       </c>
-      <c r="K60" s="69" t="s">
+      <c r="K60" s="77" t="s">
         <v>383</v>
       </c>
       <c r="L60" s="43"/>
@@ -10382,7 +10388,7 @@
       <c r="J61" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="K61" s="70"/>
+      <c r="K61" s="78"/>
       <c r="L61" s="22" t="s">
         <v>385</v>
       </c>
@@ -10422,7 +10428,7 @@
       <c r="J62" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K62" s="70"/>
+      <c r="K62" s="78"/>
       <c r="L62" s="22" t="s">
         <v>387</v>
       </c>
@@ -10462,7 +10468,7 @@
       <c r="J63" s="47" t="s">
         <v>257</v>
       </c>
-      <c r="K63" s="71"/>
+      <c r="K63" s="76"/>
       <c r="L63" s="22"/>
       <c r="M63" s="9" t="s">
         <v>257</v>
@@ -10500,7 +10506,7 @@
       <c r="J64" s="47" t="s">
         <v>257</v>
       </c>
-      <c r="K64" s="68"/>
+      <c r="K64" s="74"/>
       <c r="L64" s="22"/>
       <c r="M64" s="9" t="s">
         <v>257</v>
@@ -10538,7 +10544,7 @@
       <c r="J65" s="47" t="s">
         <v>257</v>
       </c>
-      <c r="K65" s="68"/>
+      <c r="K65" s="74"/>
       <c r="L65" s="22" t="s">
         <v>387</v>
       </c>
@@ -10576,7 +10582,7 @@
       <c r="J66" s="47" t="s">
         <v>257</v>
       </c>
-      <c r="K66" s="68"/>
+      <c r="K66" s="74"/>
       <c r="L66" s="13"/>
       <c r="M66" s="34" t="s">
         <v>257</v>
@@ -10690,7 +10696,7 @@
       <c r="J69" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K69" s="71" t="s">
+      <c r="K69" s="76" t="s">
         <v>290</v>
       </c>
       <c r="L69" s="22" t="s">
@@ -10732,7 +10738,7 @@
       <c r="J70" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K70" s="68"/>
+      <c r="K70" s="74"/>
       <c r="L70" s="22"/>
       <c r="M70" s="9" t="s">
         <v>257</v>
@@ -10810,7 +10816,7 @@
       <c r="J72" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K72" s="71"/>
+      <c r="K72" s="76"/>
       <c r="L72" s="22"/>
       <c r="M72" s="9" t="s">
         <v>257</v>
@@ -10846,7 +10852,7 @@
       <c r="J73" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K73" s="68"/>
+      <c r="K73" s="74"/>
       <c r="L73" s="22"/>
       <c r="M73" s="9" t="s">
         <v>257</v>
@@ -10882,7 +10888,7 @@
       <c r="J74" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K74" s="68"/>
+      <c r="K74" s="74"/>
       <c r="L74" s="22"/>
       <c r="M74" s="9" t="s">
         <v>257</v>
@@ -10916,7 +10922,7 @@
       <c r="J75" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K75" s="72"/>
+      <c r="K75" s="75"/>
       <c r="L75" s="44"/>
       <c r="M75" s="9" t="s">
         <v>257</v>
@@ -10994,10 +11000,10 @@
       <c r="J77" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="K77" s="80" t="s">
+      <c r="K77" s="67" t="s">
         <v>410</v>
       </c>
-      <c r="L77" s="67" t="s">
+      <c r="L77" s="73" t="s">
         <v>411</v>
       </c>
       <c r="M77" s="24" t="s">
@@ -11038,8 +11044,8 @@
       <c r="J78" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K78" s="81"/>
-      <c r="L78" s="83"/>
+      <c r="K78" s="69"/>
+      <c r="L78" s="71"/>
       <c r="M78" s="34" t="s">
         <v>257</v>
       </c>
@@ -11079,7 +11085,7 @@
       <c r="K79" s="22" t="s">
         <v>412</v>
       </c>
-      <c r="L79" s="83"/>
+      <c r="L79" s="71"/>
       <c r="M79" s="34" t="s">
         <v>257</v>
       </c>
@@ -11119,7 +11125,7 @@
       <c r="K80" s="22" t="s">
         <v>412</v>
       </c>
-      <c r="L80" s="72"/>
+      <c r="L80" s="75"/>
       <c r="M80" s="9" t="s">
         <v>257</v>
       </c>
@@ -11156,7 +11162,7 @@
       <c r="J81" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K81" s="71" t="s">
+      <c r="K81" s="76" t="s">
         <v>290</v>
       </c>
       <c r="L81" s="22" t="s">
@@ -11198,7 +11204,7 @@
       <c r="J82" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K82" s="68"/>
+      <c r="K82" s="74"/>
       <c r="L82" s="22"/>
       <c r="M82" s="9" t="s">
         <v>257</v>
@@ -11320,7 +11326,7 @@
       <c r="J85" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K85" s="71" t="s">
+      <c r="K85" s="76" t="s">
         <v>424</v>
       </c>
       <c r="L85" s="22"/>
@@ -11360,7 +11366,7 @@
       <c r="J86" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K86" s="68"/>
+      <c r="K86" s="74"/>
       <c r="L86" s="22"/>
       <c r="M86" s="9" t="s">
         <v>257</v>
@@ -11398,7 +11404,7 @@
       <c r="J87" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K87" s="68"/>
+      <c r="K87" s="74"/>
       <c r="L87" s="22"/>
       <c r="M87" s="9" t="s">
         <v>257</v>
@@ -11434,7 +11440,7 @@
       <c r="J88" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K88" s="68"/>
+      <c r="K88" s="74"/>
       <c r="L88" s="22"/>
       <c r="M88" s="9" t="s">
         <v>257</v>
@@ -11472,7 +11478,7 @@
       <c r="J89" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K89" s="68"/>
+      <c r="K89" s="74"/>
       <c r="L89" s="22"/>
       <c r="M89" s="9" t="s">
         <v>257</v>
@@ -11510,7 +11516,7 @@
       <c r="J90" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K90" s="68"/>
+      <c r="K90" s="74"/>
       <c r="L90" s="22"/>
       <c r="M90" s="9" t="s">
         <v>257</v>
@@ -11548,10 +11554,10 @@
       <c r="J91" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K91" s="80" t="s">
+      <c r="K91" s="67" t="s">
         <v>430</v>
       </c>
-      <c r="L91" s="82" t="s">
+      <c r="L91" s="70" t="s">
         <v>431</v>
       </c>
       <c r="M91" s="24" t="s">
@@ -11590,8 +11596,8 @@
       <c r="J92" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="K92" s="77"/>
-      <c r="L92" s="83"/>
+      <c r="K92" s="68"/>
+      <c r="L92" s="71"/>
       <c r="M92" s="9" t="s">
         <v>257</v>
       </c>
@@ -11628,8 +11634,8 @@
       <c r="J93" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="K93" s="77"/>
-      <c r="L93" s="83"/>
+      <c r="K93" s="68"/>
+      <c r="L93" s="71"/>
       <c r="M93" s="9" t="s">
         <v>257</v>
       </c>
@@ -11664,8 +11670,8 @@
       <c r="J94" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K94" s="81"/>
-      <c r="L94" s="84"/>
+      <c r="K94" s="69"/>
+      <c r="L94" s="72"/>
       <c r="M94" s="9" t="s">
         <v>257</v>
       </c>
@@ -11702,7 +11708,7 @@
       <c r="J95" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K95" s="67"/>
+      <c r="K95" s="73"/>
       <c r="L95" s="22"/>
       <c r="M95" s="24" t="s">
         <v>257</v>
@@ -11740,7 +11746,7 @@
       <c r="J96" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K96" s="68"/>
+      <c r="K96" s="74"/>
       <c r="L96" s="22"/>
       <c r="M96" s="24" t="s">
         <v>257</v>
@@ -11778,7 +11784,7 @@
       <c r="J97" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K97" s="68"/>
+      <c r="K97" s="74"/>
       <c r="L97" s="22"/>
       <c r="M97" s="24" t="s">
         <v>257</v>
@@ -11816,7 +11822,7 @@
       <c r="J98" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="K98" s="68"/>
+      <c r="K98" s="74"/>
       <c r="L98" s="22"/>
       <c r="M98" s="24" t="s">
         <v>257</v>
@@ -11852,7 +11858,7 @@
       <c r="J99" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="K99" s="72"/>
+      <c r="K99" s="75"/>
       <c r="L99" s="37"/>
       <c r="M99" s="39" t="s">
         <v>257</v>
@@ -11881,6 +11887,28 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="K2:K5"/>
+    <mergeCell ref="L2:L5"/>
+    <mergeCell ref="K6:K8"/>
+    <mergeCell ref="L6:L8"/>
+    <mergeCell ref="K9:K11"/>
+    <mergeCell ref="L9:L11"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="K20:K24"/>
+    <mergeCell ref="L20:L24"/>
+    <mergeCell ref="K25:K28"/>
+    <mergeCell ref="L25:L28"/>
+    <mergeCell ref="K29:K32"/>
+    <mergeCell ref="K33:K34"/>
+    <mergeCell ref="K35:K36"/>
+    <mergeCell ref="L39:L40"/>
+    <mergeCell ref="K42:K47"/>
+    <mergeCell ref="L42:L47"/>
+    <mergeCell ref="K50:K54"/>
+    <mergeCell ref="K57:K59"/>
+    <mergeCell ref="K60:K62"/>
+    <mergeCell ref="K63:K66"/>
+    <mergeCell ref="K69:K70"/>
     <mergeCell ref="K91:K94"/>
     <mergeCell ref="L91:L94"/>
     <mergeCell ref="K95:K99"/>
@@ -11889,28 +11917,6 @@
     <mergeCell ref="L77:L80"/>
     <mergeCell ref="K81:K82"/>
     <mergeCell ref="K85:K90"/>
-    <mergeCell ref="K50:K54"/>
-    <mergeCell ref="K57:K59"/>
-    <mergeCell ref="K60:K62"/>
-    <mergeCell ref="K63:K66"/>
-    <mergeCell ref="K69:K70"/>
-    <mergeCell ref="K29:K32"/>
-    <mergeCell ref="K33:K34"/>
-    <mergeCell ref="K35:K36"/>
-    <mergeCell ref="L39:L40"/>
-    <mergeCell ref="K42:K47"/>
-    <mergeCell ref="L42:L47"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="K20:K24"/>
-    <mergeCell ref="L20:L24"/>
-    <mergeCell ref="K25:K28"/>
-    <mergeCell ref="L25:L28"/>
-    <mergeCell ref="K2:K5"/>
-    <mergeCell ref="L2:L5"/>
-    <mergeCell ref="K6:K8"/>
-    <mergeCell ref="L6:L8"/>
-    <mergeCell ref="K9:K11"/>
-    <mergeCell ref="L9:L11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13060,7 +13066,9 @@
         <v>21</v>
       </c>
       <c r="H26" s="21"/>
-      <c r="I26" s="13"/>
+      <c r="I26" s="13" t="s">
+        <v>693</v>
+      </c>
       <c r="J26" s="13"/>
       <c r="K26" s="6"/>
       <c r="L26" s="6"/>
@@ -14279,7 +14287,7 @@
       </c>
       <c r="H58" s="13"/>
       <c r="I58" s="13" t="s">
-        <v>191</v>
+        <v>694</v>
       </c>
       <c r="J58" s="13"/>
       <c r="K58" s="13"/>
@@ -14312,7 +14320,7 @@
       </c>
       <c r="H59" s="13"/>
       <c r="I59" s="13" t="s">
-        <v>191</v>
+        <v>694</v>
       </c>
       <c r="J59" s="13"/>
       <c r="K59" s="13"/>

</xml_diff>